<commit_message>
Add San Miguel County openings to the job-market workbook
Nine current county postings with two salary ranges read so far: Parks and Open Space Manager at $89,316 to $100,027, and Planning Director at $116,454 to $132,175, the latter also mentioning housing. Salaries on the county board are injected by JavaScript after page load, so each has to be read from the live rendered page individually; one posting (Heavy Equipment Operator) lists no range at all. Workbook now carries four sources: seventeen weeks of print classifieds, Telski, the Town, and the County.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/Housing Study/Job Market/Telluride job market, print and employer boards.xlsx
+++ b/assets/Housing Study/Job Market/Telluride job market, print and employer boards.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method and limits" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Telski openings" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Town of Telluride openings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="County openings" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Every ad'!$A$4:$H$176</definedName>
@@ -122,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -166,6 +167,7 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -8868,4 +8870,175 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>San Miguel County, all open positions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Snapshot from the county job board on August 2, 2026. Salary appears only after the page runs its scripts, so each figure has to be read from the live page one at a time. Three have been read so far.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Position title</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Advertised pay range</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Housing mentioned</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Parks and Open Space Manager</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>$89,316 - $100,027</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Planning Director</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>$116,454 to $132,175</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Correctional Officer / Emergency Dispatcher - Telluride</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>not yet read</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Deputy Sheriff - Operations</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>not yet read</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Heavy Equipment Mechanic - Road and Bridge</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>not yet read</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Heavy Equipment Operator - Road &amp; Bridge</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>none listed</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Lead Worker - Road &amp; Bridge (Egnar)</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>not yet read</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Light Equipment Operator - Road &amp; Bridge</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>not yet read</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Senior Equipment Operator (Norwood)</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>not yet read</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>